<commit_message>
Atik kodu artik yanlislikla Sertifika Numarasi sutununa degil; P sutunundan sonra eklenen yeni Atik Kodu ve UN No sutunlarina yaziliyor
</commit_message>
<xml_diff>
--- a/bos_gonderim_sablon.xlsx
+++ b/bos_gonderim_sablon.xlsx
@@ -724,7 +724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.7109375" bestFit="1" customWidth="1" style="35" min="1" max="1"/>
@@ -743,8 +743,8 @@
     <col width="19.7109375" customWidth="1" style="35" min="14" max="14"/>
     <col width="21.7109375" customWidth="1" style="35" min="15" max="15"/>
     <col width="16.85546875" bestFit="1" customWidth="1" style="35" min="16" max="16"/>
-    <col width="15.28515625" customWidth="1" style="35" min="17" max="17"/>
-    <col width="26" customWidth="1" style="35" min="18" max="18"/>
+    <col width="22" customWidth="1" style="35" min="17" max="17"/>
+    <col width="18" customWidth="1" style="35" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -768,12 +768,12 @@
       <c r="N1" s="45" t="n"/>
       <c r="O1" s="45" t="n"/>
       <c r="P1" s="46" t="n"/>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Doküman No: </t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>TMGDK-L2</t>
         </is>
@@ -795,12 +795,12 @@
       <c r="N2" s="51" t="n"/>
       <c r="O2" s="51" t="n"/>
       <c r="P2" s="52" t="n"/>
-      <c r="Q2" s="7" t="inlineStr">
+      <c r="S2" s="7" t="inlineStr">
         <is>
           <t>Yayın Tarihi:</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>31.11.2024</t>
         </is>
@@ -826,12 +826,12 @@
       <c r="N3" s="45" t="n"/>
       <c r="O3" s="45" t="n"/>
       <c r="P3" s="46" t="n"/>
-      <c r="Q3" s="7" t="inlineStr">
+      <c r="S3" s="7" t="inlineStr">
         <is>
           <t>Revizyon Tarihi:</t>
         </is>
       </c>
-      <c r="R3" s="2" t="n">
+      <c r="T3" s="2" t="n">
         <v>46192</v>
       </c>
     </row>
@@ -852,12 +852,12 @@
       <c r="N4" s="51" t="n"/>
       <c r="O4" s="51" t="n"/>
       <c r="P4" s="52" t="n"/>
-      <c r="Q4" s="7" t="inlineStr">
+      <c r="S4" s="7" t="inlineStr">
         <is>
           <t>Sayfa No:</t>
         </is>
       </c>
-      <c r="R4" s="17" t="n"/>
+      <c r="T4" s="17" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -942,10 +942,20 @@
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
+          <t>Atık Kodu</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>UN No</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
           <t>Yük Miktarı (KG)</t>
         </is>
       </c>
-      <c r="R5" s="8" t="inlineStr">
+      <c r="T5" s="8" t="inlineStr">
         <is>
           <t>Kontrol Formunu Dolduran Kişi</t>
         </is>

</xml_diff>